<commit_message>
060425 - updated skins spreadsheet format
</commit_message>
<xml_diff>
--- a/public/results/2025/Week 2 Skins.xlsx
+++ b/public/results/2025/Week 2 Skins.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98B3A5E4-D3B2-6544-ABE4-3AD9661E52D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790A2912-D09C-E44B-9F36-265F855121BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{649A485E-B014-E445-AC7D-E025E3369B85}"/>
   </bookViews>
@@ -38,9 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="31">
   <si>
-    <t>Name (skins won)</t>
-  </si>
-  <si>
     <t>Actual</t>
   </si>
   <si>
@@ -129,6 +126,9 @@
   </si>
   <si>
     <t>Shayne</t>
+  </si>
+  <si>
+    <t>Skins Won</t>
   </si>
 </sst>
 </file>
@@ -903,6 +903,7 @@
   <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="14.5" customWidth="1"/>
     <col min="2" max="2" width="8.5" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
     <col min="4" max="4" width="2.6640625" customWidth="1"/>
@@ -911,18 +912,18 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" s="4"/>
       <c r="E1" s="5"/>
       <c r="F1" s="6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G1" s="6">
         <v>4</v>
@@ -954,7 +955,7 @@
     </row>
     <row r="2" spans="1:15" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="9">
         <v>19.98</v>
@@ -965,7 +966,7 @@
       <c r="D2" s="11"/>
       <c r="E2" s="5"/>
       <c r="F2" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G2" s="12">
         <v>4</v>
@@ -997,7 +998,7 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" s="9">
         <v>8.8800000000000008</v>
@@ -1007,7 +1008,7 @@
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" s="14">
         <v>13</v>
@@ -1042,7 +1043,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="9">
         <v>2.2200000000000002</v>
@@ -1053,7 +1054,7 @@
       <c r="D4" s="11"/>
       <c r="E4" s="15"/>
       <c r="F4" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G4" s="16">
         <v>2</v>
@@ -1085,7 +1086,7 @@
     </row>
     <row r="5" spans="1:15" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="9">
         <v>2.2200000000000002</v>
@@ -1096,7 +1097,7 @@
       <c r="D5" s="11"/>
       <c r="E5" s="15"/>
       <c r="F5" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G5" s="17">
         <v>3</v>
@@ -1128,7 +1129,7 @@
     </row>
     <row r="6" spans="1:15" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" s="22">
         <v>2.2200000000000002</v>
@@ -1138,7 +1139,7 @@
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" s="14">
         <v>8</v>
@@ -1173,7 +1174,7 @@
     </row>
     <row r="7" spans="1:15" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="25">
         <f>SUM(B2:B6)</f>
@@ -1185,7 +1186,7 @@
       <c r="D7" s="11"/>
       <c r="E7" s="15"/>
       <c r="F7" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G7" s="16">
         <v>1</v>
@@ -1220,7 +1221,7 @@
       <c r="D8" s="28"/>
       <c r="E8" s="15"/>
       <c r="F8" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G8" s="18">
         <v>6</v>
@@ -1256,7 +1257,7 @@
       <c r="C9" s="27"/>
       <c r="D9" s="28"/>
       <c r="E9" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F9" s="14">
         <v>17</v>
@@ -1296,7 +1297,7 @@
       <c r="D10" s="28"/>
       <c r="E10" s="15"/>
       <c r="F10" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G10" s="16">
         <v>2</v>
@@ -1333,7 +1334,7 @@
       <c r="D11" s="28"/>
       <c r="E11" s="15"/>
       <c r="F11" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G11" s="18">
         <v>5</v>
@@ -1369,7 +1370,7 @@
       <c r="C12" s="27"/>
       <c r="D12" s="28"/>
       <c r="E12" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F12" s="14">
         <v>21</v>
@@ -1409,7 +1410,7 @@
       <c r="D13" s="28"/>
       <c r="E13" s="15"/>
       <c r="F13" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G13" s="16">
         <v>2</v>
@@ -1446,7 +1447,7 @@
       <c r="D14" s="28"/>
       <c r="E14" s="15"/>
       <c r="F14" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G14" s="18">
         <v>6</v>
@@ -1482,7 +1483,7 @@
       <c r="C15" s="27"/>
       <c r="D15" s="28"/>
       <c r="E15" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F15" s="14">
         <v>15</v>
@@ -1522,7 +1523,7 @@
       <c r="D16" s="28"/>
       <c r="E16" s="15"/>
       <c r="F16" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G16" s="16">
         <v>2</v>
@@ -1559,7 +1560,7 @@
       <c r="D17" s="28"/>
       <c r="E17" s="15"/>
       <c r="F17" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G17" s="18">
         <v>5</v>
@@ -1595,7 +1596,7 @@
       <c r="C18" s="27"/>
       <c r="D18" s="28"/>
       <c r="E18" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F18" s="14">
         <v>22</v>
@@ -1635,7 +1636,7 @@
       <c r="D19" s="28"/>
       <c r="E19" s="15"/>
       <c r="F19" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G19" s="16">
         <v>3</v>
@@ -1672,7 +1673,7 @@
       <c r="D20" s="28"/>
       <c r="E20" s="15"/>
       <c r="F20" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G20" s="17">
         <v>3</v>
@@ -1708,7 +1709,7 @@
       <c r="C21" s="27"/>
       <c r="D21" s="28"/>
       <c r="E21" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F21" s="14">
         <v>18</v>
@@ -1748,7 +1749,7 @@
       <c r="D22" s="28"/>
       <c r="E22" s="15"/>
       <c r="F22" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G22" s="16">
         <v>2</v>
@@ -1785,7 +1786,7 @@
       <c r="D23" s="28"/>
       <c r="E23" s="15"/>
       <c r="F23" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G23" s="17">
         <v>3</v>
@@ -1821,7 +1822,7 @@
       <c r="C24" s="27"/>
       <c r="D24" s="28"/>
       <c r="E24" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F24" s="14">
         <v>8</v>
@@ -1861,7 +1862,7 @@
       <c r="D25" s="28"/>
       <c r="E25" s="28"/>
       <c r="F25" s="28" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G25" s="27">
         <v>1</v>
@@ -1896,7 +1897,7 @@
       <c r="D26" s="28"/>
       <c r="E26" s="28"/>
       <c r="F26" s="28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G26" s="30">
         <v>4</v>
@@ -1951,31 +1952,31 @@
       <c r="E28" s="28"/>
       <c r="F28" s="28"/>
       <c r="G28" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="H28" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="H28" s="27" t="s">
+      <c r="I28" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="27" t="s">
+      <c r="J28" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="K28" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="J28" s="27" t="s">
+      <c r="L28" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="K28" s="29" t="s">
+      <c r="M28" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="N28" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="O28" s="29" t="s">
         <v>24</v>
-      </c>
-      <c r="L28" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="M28" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="N28" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="O28" s="29" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
@@ -1987,25 +1988,25 @@
       <c r="F29" s="28"/>
       <c r="G29" s="27"/>
       <c r="H29" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="I29" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="I29" s="27" t="s">
+      <c r="J29" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="K29" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="L29" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="J29" s="27" t="s">
+      <c r="M29" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K29" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="L29" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="M29" s="29" t="s">
-        <v>27</v>
-      </c>
       <c r="N29" s="29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O29" s="29"/>
     </row>
@@ -2052,10 +2053,10 @@
       <c r="I31" s="27"/>
       <c r="J31" s="27"/>
       <c r="K31" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="L31" s="29" t="s">
         <v>29</v>
-      </c>
-      <c r="L31" s="29" t="s">
-        <v>30</v>
       </c>
       <c r="M31" s="29"/>
       <c r="N31" s="29"/>

</xml_diff>